<commit_message>
Dashboard update 2026-08-03 21:31
</commit_message>
<xml_diff>
--- a/excel/Lendermarket.xlsx
+++ b/excel/Lendermarket.xlsx
@@ -1,33 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Investavimas 2026.06.03\Lendermarket\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.06.03\Lendermarket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54492164-CD85-4A5B-B1A0-C8554E4F0527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1FA814D-6A6D-4ACB-9E78-2027C3816B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
     <sheet name="Pinigai" sheetId="15" r:id="rId2"/>
-    <sheet name="8945000DP4C3YFA45N3453716086" sheetId="30" r:id="rId3"/>
-    <sheet name="8945000DP4C3YFA45N3469604165" sheetId="29" r:id="rId4"/>
-    <sheet name="8945000DP4C3YFA45N3460847714" sheetId="28" r:id="rId5"/>
-    <sheet name="8945000DP4C3YFA45N3489849864" sheetId="27" r:id="rId6"/>
-    <sheet name="8945000DP4C3YFA45N3431128353" sheetId="26" r:id="rId7"/>
-    <sheet name="8945000DP4C3YFA45N3430165789" sheetId="25" r:id="rId8"/>
-    <sheet name="8945000DP4C3YFA45N3432815787" sheetId="24" r:id="rId9"/>
-    <sheet name="8945000DP4C3YFA45N3413372056" sheetId="23" r:id="rId10"/>
-    <sheet name="8945000DP4C3YFA45N3413742182" sheetId="22" r:id="rId11"/>
-    <sheet name="8945000DP4C3YFA45N3480247173" sheetId="21" r:id="rId12"/>
-    <sheet name="8945000DP4C3YFA45N3431985084" sheetId="20" r:id="rId13"/>
-    <sheet name="8945000DP4C3YFA45N3421733887" sheetId="19" r:id="rId14"/>
-    <sheet name="de81-49b6-a7b5-77be994b7d06" sheetId="18" r:id="rId15"/>
+    <sheet name="8945000DP4C3YFA45N3457082561" sheetId="31" r:id="rId3"/>
+    <sheet name="8945000DP4C3YFA45N3453716086" sheetId="30" r:id="rId4"/>
+    <sheet name="8945000DP4C3YFA45N3469604165" sheetId="29" r:id="rId5"/>
+    <sheet name="8945000DP4C3YFA45N3460847714" sheetId="28" r:id="rId6"/>
+    <sheet name="8945000DP4C3YFA45N3489849864" sheetId="27" r:id="rId7"/>
+    <sheet name="8945000DP4C3YFA45N3431128353" sheetId="26" r:id="rId8"/>
+    <sheet name="8945000DP4C3YFA45N3430165789" sheetId="25" r:id="rId9"/>
+    <sheet name="8945000DP4C3YFA45N3432815787" sheetId="24" r:id="rId10"/>
+    <sheet name="8945000DP4C3YFA45N3413372056" sheetId="23" r:id="rId11"/>
+    <sheet name="8945000DP4C3YFA45N3413742182" sheetId="22" r:id="rId12"/>
+    <sheet name="8945000DP4C3YFA45N3480247173" sheetId="21" r:id="rId13"/>
+    <sheet name="8945000DP4C3YFA45N3431985084" sheetId="20" r:id="rId14"/>
+    <sheet name="8945000DP4C3YFA45N3421733887" sheetId="19" r:id="rId15"/>
+    <sheet name="de81-49b6-a7b5-77be994b7d06" sheetId="18" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="69">
   <si>
     <t>Paskola</t>
   </si>
@@ -248,6 +249,15 @@
   </si>
   <si>
     <t xml:space="preserve">Premijos </t>
+  </si>
+  <si>
+    <t>8945000DP4C3YFA45N3457082561</t>
+  </si>
+  <si>
+    <t>Colombia</t>
+  </si>
+  <si>
+    <t>Rapicredit</t>
   </si>
 </sst>
 </file>
@@ -500,7 +510,35 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="56">
+  <dxfs count="60">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -927,7 +965,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C5054642-0730-4BCF-95E8-D8A572C38E82}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E87D4FA7-1EB5-414A-B5B5-7CD81172CD32}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -983,7 +1021,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C1C4A01-D049-4E52-9648-88D269C70B9A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B9728F8C-AFD4-4C72-B65C-67D97C1D5A17}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1039,7 +1077,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42B31D62-7349-472B-8B1B-60B1E044FF6F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C1C4A01-D049-4E52-9648-88D269C70B9A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1095,6 +1133,62 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42B31D62-7349-472B-8B1B-60B1E044FF6F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId3"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="3619500"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>914400</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Graphic 1" descr="Arrow: Rotate left with solid fill">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD32E591-CDB5-4E6C-848C-6BC9193D2605}"/>
             </a:ext>
           </a:extLst>
@@ -1130,7 +1224,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1207,7 +1301,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4049674A-AB09-4980-A167-42707A5C065E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C5054642-0730-4BCF-95E8-D8A572C38E82}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1263,7 +1357,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5D16B82-4527-4AC8-BE2C-F18ECB083711}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4049674A-AB09-4980-A167-42707A5C065E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1319,7 +1413,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED5BAA2D-5804-48F9-96B5-DD2F9A5952EE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5D16B82-4527-4AC8-BE2C-F18ECB083711}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1375,7 +1469,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62154965-B37D-4F49-8A1B-F820A3B2DD47}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED5BAA2D-5804-48F9-96B5-DD2F9A5952EE}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1431,7 +1525,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B739419F-97B7-4047-BD1E-CEA0E8CF25ED}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62154965-B37D-4F49-8A1B-F820A3B2DD47}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1487,7 +1581,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0F9F9B1D-4F5D-4A37-9402-DCF282E8ABF5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B739419F-97B7-4047-BD1E-CEA0E8CF25ED}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1543,7 +1637,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF165EBA-6D1B-498D-B7F3-F18C63C99360}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0F9F9B1D-4F5D-4A37-9402-DCF282E8ABF5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1599,7 +1693,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B9728F8C-AFD4-4C72-B65C-67D97C1D5A17}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF165EBA-6D1B-498D-B7F3-F18C63C99360}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2081,7 +2175,7 @@
       </c>
       <c r="K3" s="16">
         <f ca="1">'de81-49b6-a7b5-77be994b7d06'!B12</f>
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="L3" s="16" t="str">
         <f ca="1">'de81-49b6-a7b5-77be994b7d06'!P3</f>
@@ -2106,7 +2200,7 @@
       </c>
       <c r="R3" s="29">
         <f>SUM(H3:H100)-U3</f>
-        <v>105.44</v>
+        <v>111.90999999999998</v>
       </c>
       <c r="S3" s="28">
         <f>Pinigai!H2</f>
@@ -2114,31 +2208,31 @@
       </c>
       <c r="T3" s="28">
         <f>W3-R3</f>
-        <v>6.3500000000000085</v>
+        <v>0</v>
       </c>
       <c r="U3" s="29">
         <f>SUM(M3:M100)</f>
-        <v>57.199999999999996</v>
+        <v>61.429999999999993</v>
       </c>
       <c r="V3" s="29">
         <f>SUM(N3:N100)-AA3</f>
-        <v>1.34</v>
+        <v>1.46</v>
       </c>
       <c r="W3" s="28">
         <f>Q3+S3+V3</f>
-        <v>111.79</v>
+        <v>111.91</v>
       </c>
       <c r="X3" s="28">
         <f>W3-Q3</f>
-        <v>11.790000000000006</v>
+        <v>11.909999999999997</v>
       </c>
       <c r="Y3" s="30">
         <f>(W3-Q3)/Q3</f>
-        <v>0.11790000000000006</v>
+        <v>0.11909999999999997</v>
       </c>
       <c r="Z3" s="31">
         <f ca="1">XIRR(Pinigai!K3:K200,Pinigai!A3:A200)</f>
-        <v>1.1068951487541201</v>
+        <v>1.0414577364921571</v>
       </c>
       <c r="AA3" s="28">
         <f>SUM(O3:O100)</f>
@@ -2191,7 +2285,7 @@
       </c>
       <c r="K4" s="16">
         <f ca="1">'8945000DP4C3YFA45N3421733887'!B12</f>
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="L4" s="16" t="str">
         <f ca="1">'8945000DP4C3YFA45N3421733887'!P3</f>
@@ -2399,7 +2493,7 @@
       </c>
       <c r="K7" s="16">
         <f ca="1">'8945000DP4C3YFA45N3413742182'!B12</f>
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="L7" s="16" t="str">
         <f ca="1">'8945000DP4C3YFA45N3413742182'!P3</f>
@@ -2465,7 +2559,7 @@
       </c>
       <c r="K8" s="16">
         <f ca="1">'8945000DP4C3YFA45N3413372056'!B12</f>
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="L8" s="16" t="str">
         <f ca="1">'8945000DP4C3YFA45N3413372056'!P3</f>
@@ -2597,7 +2691,7 @@
       </c>
       <c r="K10" s="16">
         <f ca="1">'8945000DP4C3YFA45N3430165789'!B12</f>
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L10" s="16" t="str">
         <f ca="1">'8945000DP4C3YFA45N3430165789'!P3</f>
@@ -2605,11 +2699,11 @@
       </c>
       <c r="M10" s="3">
         <f>'8945000DP4C3YFA45N3430165789'!K3</f>
-        <v>3.19</v>
+        <v>6.41</v>
       </c>
       <c r="N10" s="3">
         <f>'8945000DP4C3YFA45N3430165789'!L3</f>
-        <v>0.05</v>
+        <v>0.13</v>
       </c>
       <c r="O10" s="3">
         <f>'8945000DP4C3YFA45N3430165789'!M3</f>
@@ -2663,7 +2757,7 @@
       </c>
       <c r="K11" s="16">
         <f ca="1">'8945000DP4C3YFA45N3431128353'!B12</f>
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="L11" s="16" t="str">
         <f ca="1">'8945000DP4C3YFA45N3431128353'!P3</f>
@@ -2729,11 +2823,11 @@
       </c>
       <c r="K12" s="16">
         <f ca="1">'8945000DP4C3YFA45N3489849864'!B12</f>
-        <v>-6</v>
+        <v>-9</v>
       </c>
       <c r="L12" s="16">
         <f ca="1">'8945000DP4C3YFA45N3489849864'!P3</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M12" s="3">
         <f>'8945000DP4C3YFA45N3489849864'!K3</f>
@@ -2794,7 +2888,7 @@
       </c>
       <c r="K13" s="16">
         <f ca="1">'8945000DP4C3YFA45N3460847714'!B12</f>
-        <v>1242</v>
+        <v>1239</v>
       </c>
       <c r="L13" s="16" t="str">
         <f ca="1">'8945000DP4C3YFA45N3460847714'!P3</f>
@@ -2859,7 +2953,7 @@
       </c>
       <c r="K14" s="16">
         <f ca="1">'8945000DP4C3YFA45N3469604165'!B12</f>
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="L14" s="16" t="str">
         <f ca="1">'8945000DP4C3YFA45N3469604165'!P3</f>
@@ -2924,7 +3018,7 @@
       </c>
       <c r="K15" s="16">
         <f ca="1">'8945000DP4C3YFA45N3453716086'!B12</f>
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="L15" s="16" t="str">
         <f ca="1">'8945000DP4C3YFA45N3453716086'!P3</f>
@@ -2932,11 +3026,11 @@
       </c>
       <c r="M15" s="3">
         <f>'8945000DP4C3YFA45N3453716086'!K3</f>
-        <v>0</v>
+        <v>1.01</v>
       </c>
       <c r="N15" s="3">
         <f>'8945000DP4C3YFA45N3453716086'!L3</f>
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="O15" s="3">
         <f>'8945000DP4C3YFA45N3453716086'!M3</f>
@@ -2948,22 +3042,69 @@
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="AC16" s="1"/>
+      <c r="A16" s="2">
+        <v>14</v>
+      </c>
+      <c r="B16" s="6">
+        <f>'8945000DP4C3YFA45N3457082561'!B9</f>
+        <v>46234</v>
+      </c>
+      <c r="C16" s="15" t="str">
+        <f>'8945000DP4C3YFA45N3457082561'!B1</f>
+        <v>8945000DP4C3YFA45N3457082561</v>
+      </c>
+      <c r="D16" s="2" t="str">
+        <f>'8945000DP4C3YFA45N3457082561'!B2</f>
+        <v>Colombia</v>
+      </c>
+      <c r="E16" s="2" t="str">
+        <f>'8945000DP4C3YFA45N3457082561'!B3</f>
+        <v>Rapicredit</v>
+      </c>
+      <c r="F16" s="2" t="str">
+        <f>'8945000DP4C3YFA45N3457082561'!B8</f>
+        <v>0 m. 2 mėn. 12 d.</v>
+      </c>
+      <c r="G16" s="7">
+        <f>'8945000DP4C3YFA45N3457082561'!B15</f>
+        <v>0.15</v>
+      </c>
+      <c r="H16" s="3">
+        <f>'8945000DP4C3YFA45N3457082561'!B16</f>
+        <v>10.7</v>
+      </c>
+      <c r="I16" s="6">
+        <f>'8945000DP4C3YFA45N3457082561'!B11</f>
+        <v>46308</v>
+      </c>
+      <c r="J16" s="6" t="str">
+        <f>'8945000DP4C3YFA45N3457082561'!O3</f>
+        <v/>
+      </c>
+      <c r="K16" s="16">
+        <f ca="1">'8945000DP4C3YFA45N3457082561'!B12</f>
+        <v>73</v>
+      </c>
+      <c r="L16" s="16" t="str">
+        <f ca="1">'8945000DP4C3YFA45N3457082561'!P3</f>
+        <v/>
+      </c>
+      <c r="M16" s="3">
+        <f>'8945000DP4C3YFA45N3457082561'!K3</f>
+        <v>0</v>
+      </c>
+      <c r="N16" s="3">
+        <f>'8945000DP4C3YFA45N3457082561'!L3</f>
+        <v>0</v>
+      </c>
+      <c r="O16" s="3">
+        <f>'8945000DP4C3YFA45N3457082561'!M3</f>
+        <v>0</v>
+      </c>
+      <c r="AC16" s="3" t="str">
+        <f ca="1">'8945000DP4C3YFA45N3457082561'!Z3</f>
+        <v/>
+      </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
@@ -3173,18 +3314,18 @@
     <mergeCell ref="U1:V1"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:O27">
-    <cfRule type="expression" dxfId="55" priority="12">
+    <cfRule type="expression" dxfId="59" priority="14">
       <formula>$AC3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="54" priority="13">
+    <cfRule type="expression" dxfId="58" priority="15">
       <formula>AND($M3&gt;0,$H3=$M3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC3:AC27">
-    <cfRule type="expression" dxfId="53" priority="1">
+    <cfRule type="expression" dxfId="57" priority="1">
       <formula>$AC3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="52" priority="2">
+    <cfRule type="expression" dxfId="56" priority="2">
       <formula>AND($M3&gt;0,$H3=$M3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3202,6 +3343,7 @@
     <hyperlink ref="C13" location="'8945000DP4C3YFA45N3460847714'!A1" display="'8945000DP4C3YFA45N3460847714'!A1" xr:uid="{5771895D-B06F-4E31-9E5E-950B34460F21}"/>
     <hyperlink ref="C14" location="'8945000DP4C3YFA45N3469604165'!A1" display="'8945000DP4C3YFA45N3469604165'!A1" xr:uid="{A999F8E1-D281-4667-BB59-66D7839421D7}"/>
     <hyperlink ref="C15" location="'8945000DP4C3YFA45N3453716086'!A1" display="'8945000DP4C3YFA45N3453716086'!A1" xr:uid="{6FA669DF-4A4F-4C46-BBF1-79DE5405B382}"/>
+    <hyperlink ref="C16" location="'8945000DP4C3YFA45N3457082561'!A1" display="'8945000DP4C3YFA45N3457082561'!A1" xr:uid="{CD357B36-E437-4FAF-84E0-F5C1113D1CE3}"/>
   </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="50" orientation="landscape" r:id="rId1"/>
@@ -3209,6 +3351,1311 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{615F6B81-524E-46B8-96DD-07557B282857}">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:Z53"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="40.7109375" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" customWidth="1"/>
+    <col min="11" max="14" width="10.7109375" customWidth="1"/>
+    <col min="15" max="15" width="12.7109375" customWidth="1"/>
+    <col min="16" max="17" width="10.7109375" customWidth="1"/>
+    <col min="18" max="23" width="8.7109375" customWidth="1"/>
+    <col min="24" max="24" width="12.7109375" style="13" customWidth="1"/>
+    <col min="25" max="25" width="10.7109375" style="13" customWidth="1"/>
+    <col min="26" max="26" width="10.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="33"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="32" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="33"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33"/>
+      <c r="P1" s="33"/>
+      <c r="Q1" s="34"/>
+      <c r="X1" s="32"/>
+      <c r="Y1" s="33"/>
+      <c r="Z1" s="34"/>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="9"/>
+      <c r="K2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="M2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="X2" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="Y2" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z2" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="10">
+        <v>46172</v>
+      </c>
+      <c r="E3" s="10">
+        <v>46174</v>
+      </c>
+      <c r="F3" s="16">
+        <f>IF(E3&gt;0,E3-D3,"")</f>
+        <v>2</v>
+      </c>
+      <c r="G3" s="3">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
+      <c r="J3" s="13"/>
+      <c r="K3" s="3">
+        <f>G53</f>
+        <v>12.809999999999999</v>
+      </c>
+      <c r="L3" s="3">
+        <f>H53</f>
+        <v>0.11</v>
+      </c>
+      <c r="M3" s="3">
+        <f>I53</f>
+        <v>0</v>
+      </c>
+      <c r="N3" s="7">
+        <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
+        <v>0.11385952830314636</v>
+      </c>
+      <c r="O3" s="6">
+        <f>IF(B16=K3,MAX(E:E),"")</f>
+        <v>46205</v>
+      </c>
+      <c r="P3" s="2" t="str">
+        <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
+        <v/>
+      </c>
+      <c r="Q3" s="2">
+        <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
+        <v>-271</v>
+      </c>
+      <c r="T3" s="12"/>
+      <c r="X3" s="6">
+        <f>B9</f>
+        <v>46169</v>
+      </c>
+      <c r="Y3" s="3">
+        <f>B16*-1</f>
+        <v>-12.81</v>
+      </c>
+      <c r="Z3" s="2" t="str">
+        <f ca="1">IF(AND(TODAY()&gt;B11, K3&lt;&gt;B16), "+", "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="10">
+        <v>46203</v>
+      </c>
+      <c r="E4" s="10">
+        <v>46175</v>
+      </c>
+      <c r="F4" s="16">
+        <f>IF(E4&gt;0,E4-D4,"")</f>
+        <v>-28</v>
+      </c>
+      <c r="G4" s="3">
+        <v>1.81</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="I4" s="3">
+        <v>0</v>
+      </c>
+      <c r="J4" s="9"/>
+      <c r="X4" s="6">
+        <f>E3</f>
+        <v>46174</v>
+      </c>
+      <c r="Y4" s="3">
+        <f>G3+H3-I3</f>
+        <v>1.17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A5" s="5"/>
+      <c r="B5" s="6"/>
+      <c r="D5" s="10">
+        <v>46233</v>
+      </c>
+      <c r="E5" s="10">
+        <v>46205</v>
+      </c>
+      <c r="F5" s="16">
+        <f t="shared" ref="F5:F52" si="0">IF(E5&gt;0,E5-D5,"")</f>
+        <v>-28</v>
+      </c>
+      <c r="G5" s="3">
+        <v>9.84</v>
+      </c>
+      <c r="H5" s="3">
+        <v>0.09</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9"/>
+      <c r="X5" s="6">
+        <f t="shared" ref="X5:X52" si="1">E4</f>
+        <v>46175</v>
+      </c>
+      <c r="Y5" s="3">
+        <f t="shared" ref="Y5:Y52" si="2">G4+H4-I4</f>
+        <v>1.82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A6" s="5"/>
+      <c r="B6" s="6"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="9"/>
+      <c r="X6" s="6">
+        <f t="shared" si="1"/>
+        <v>46205</v>
+      </c>
+      <c r="Y6" s="3">
+        <f t="shared" si="2"/>
+        <v>9.93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A7" s="5"/>
+      <c r="B7" s="6"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="13"/>
+      <c r="X7" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y7" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="6" t="str">
+        <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
+        <v>0 m. 10 mėn. 3 d.</v>
+      </c>
+      <c r="D8" s="10"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="9"/>
+      <c r="X8" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y8" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="6">
+        <v>46169</v>
+      </c>
+      <c r="D9" s="10"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="13"/>
+      <c r="X9" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y9" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="6">
+        <v>46108</v>
+      </c>
+      <c r="D10" s="10"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="13"/>
+      <c r="X10" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y10" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="6">
+        <v>46476</v>
+      </c>
+      <c r="D11" s="10"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="13"/>
+      <c r="X11" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y11" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="16" t="str">
+        <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
+        <v/>
+      </c>
+      <c r="D12" s="10"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="13"/>
+      <c r="X12" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y12" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A13" s="5"/>
+      <c r="B13" s="3"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="13"/>
+      <c r="N13" s="12"/>
+      <c r="X13" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y13" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="22"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="13"/>
+      <c r="X14" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y14" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="7">
+        <v>0.11</v>
+      </c>
+      <c r="D15" s="10"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="18"/>
+      <c r="M15" s="18"/>
+      <c r="N15" s="18"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="18"/>
+      <c r="Q15" s="18"/>
+      <c r="X15" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y15" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="3">
+        <v>12.81</v>
+      </c>
+      <c r="D16" s="10"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="19"/>
+      <c r="O16" s="20"/>
+      <c r="P16" s="13"/>
+      <c r="Q16" s="13"/>
+      <c r="X16" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y16" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D17" s="10"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="13"/>
+      <c r="X17" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y17" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D18" s="10"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="13"/>
+      <c r="X18" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y18" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D19" s="10"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="13"/>
+      <c r="X19" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y19" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D20" s="10"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="13"/>
+      <c r="X20" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y20" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D21" s="10"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="13"/>
+      <c r="X21" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y21" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D22" s="10"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="13"/>
+      <c r="X22" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y22" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D23" s="10"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="13"/>
+      <c r="X23" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y23" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D24" s="10"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="13"/>
+      <c r="X24" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y24" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D25" s="10"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="13"/>
+      <c r="X25" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y25" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D26" s="10"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="13"/>
+      <c r="X26" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y26" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D27" s="10"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="13"/>
+      <c r="X27" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y27" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D28" s="10"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="13"/>
+      <c r="X28" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y28" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D29" s="10"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="13"/>
+      <c r="X29" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y29" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D30" s="10"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="13"/>
+      <c r="X30" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y30" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D31" s="10"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="13"/>
+      <c r="X31" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y31" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D32" s="10"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="13"/>
+      <c r="X32" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y32" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D33" s="10"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="13"/>
+      <c r="X33" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y33" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D34" s="10"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="13"/>
+      <c r="X34" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y34" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D35" s="10"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="13"/>
+      <c r="X35" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y35" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D36" s="10"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="13"/>
+      <c r="X36" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y36" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D37" s="10"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="13"/>
+      <c r="X37" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y37" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D38" s="10"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="13"/>
+      <c r="X38" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y38" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D39" s="10"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="13"/>
+      <c r="X39" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y39" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D40" s="10"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="13"/>
+      <c r="X40" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y40" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D41" s="10"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="13"/>
+      <c r="X41" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y41" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D42" s="10"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="13"/>
+      <c r="X42" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y42" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D43" s="10"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
+      <c r="J43" s="13"/>
+      <c r="X43" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y43" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D44" s="10"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="13"/>
+      <c r="X44" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y44" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D45" s="10"/>
+      <c r="E45" s="6"/>
+      <c r="F45" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="13"/>
+      <c r="X45" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y45" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D46" s="10"/>
+      <c r="E46" s="6"/>
+      <c r="F46" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2"/>
+      <c r="J46" s="13"/>
+      <c r="X46" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y46" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D47" s="10"/>
+      <c r="E47" s="6"/>
+      <c r="F47" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+      <c r="J47" s="13"/>
+      <c r="X47" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y47" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D48" s="10"/>
+      <c r="E48" s="6"/>
+      <c r="F48" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="13"/>
+      <c r="X48" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y48" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D49" s="10"/>
+      <c r="E49" s="6"/>
+      <c r="F49" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
+      <c r="I49" s="2"/>
+      <c r="J49" s="13"/>
+      <c r="X49" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y49" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D50" s="10"/>
+      <c r="E50" s="6"/>
+      <c r="F50" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
+      <c r="I50" s="2"/>
+      <c r="J50" s="13"/>
+      <c r="X50" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y50" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D51" s="10"/>
+      <c r="E51" s="6"/>
+      <c r="F51" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="13"/>
+      <c r="X51" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y51" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D52" s="10"/>
+      <c r="E52" s="6"/>
+      <c r="F52" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="9"/>
+      <c r="X52" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y52" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D53" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E53" s="23"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3">
+        <f>SUM(G3:G52)</f>
+        <v>12.809999999999999</v>
+      </c>
+      <c r="H53" s="3">
+        <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
+        <v>0.11</v>
+      </c>
+      <c r="I53" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="K1:Q1"/>
+    <mergeCell ref="X1:Z1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1:B1">
+    <cfRule type="expression" dxfId="27" priority="1">
+      <formula>$Z$3="+"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="26" priority="2">
+      <formula>$B$16=$K$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P3">
+    <cfRule type="expression" dxfId="25" priority="5">
+      <formula>$Z$3="+"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z3">
+    <cfRule type="expression" dxfId="24" priority="6">
+      <formula>$Z$3="+"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0217942-24E3-4183-AA84-999E51E414ED}">
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3600,7 +5047,7 @@
       </c>
       <c r="B12" s="16">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -4502,7 +5949,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD4BDDE2-8704-4234-A130-5A9141225661}">
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4750,7 +6197,9 @@
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="6"/>
-      <c r="D6" s="10"/>
+      <c r="D6" s="10">
+        <v>46261</v>
+      </c>
       <c r="E6" s="10"/>
       <c r="F6" s="16" t="str">
         <f t="shared" si="0"/>
@@ -4902,7 +6351,7 @@
       </c>
       <c r="B12" s="16">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -5804,7 +7253,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DB3AF2E-D350-415A-BB99-2F8DABB3126C}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -7089,7 +8538,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AF1F64B-FA87-4FC9-BBF4-0658CCF42B49}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -8374,7 +9823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E29E82-AEB9-428A-AE0E-F12CE0B61744}">
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8786,7 +10235,7 @@
       </c>
       <c r="B12" s="16">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -9688,7 +11137,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCFE81BF-3088-410D-89E1-7093256A7CF9}">
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10100,7 +11549,7 @@
       </c>
       <c r="B12" s="16">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -12589,14 +14038,14 @@
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200" s="6">
         <f ca="1">TODAY()</f>
-        <v>46232</v>
+        <v>46235</v>
       </c>
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
       <c r="D200" s="1"/>
       <c r="K200" s="3">
         <f>Overview!W3</f>
-        <v>111.79</v>
+        <v>111.91</v>
       </c>
     </row>
   </sheetData>
@@ -12606,6 +14055,1282 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93F1ED2E-BBE4-425E-B774-C63E5954DB79}">
+  <dimension ref="A1:Z53"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="40.7109375" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" customWidth="1"/>
+    <col min="11" max="14" width="10.7109375" customWidth="1"/>
+    <col min="15" max="15" width="12.7109375" customWidth="1"/>
+    <col min="16" max="17" width="10.7109375" customWidth="1"/>
+    <col min="18" max="23" width="8.7109375" customWidth="1"/>
+    <col min="24" max="24" width="12.7109375" style="13" customWidth="1"/>
+    <col min="25" max="25" width="10.7109375" style="13" customWidth="1"/>
+    <col min="26" max="26" width="10.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="33"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="32" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="33"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33"/>
+      <c r="P1" s="33"/>
+      <c r="Q1" s="34"/>
+      <c r="X1" s="32"/>
+      <c r="Y1" s="33"/>
+      <c r="Z1" s="34"/>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="9"/>
+      <c r="K2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="M2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="X2" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="Y2" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z2" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="10">
+        <v>46308</v>
+      </c>
+      <c r="E3" s="10"/>
+      <c r="F3" s="16" t="str">
+        <f>IF(E3&gt;0,E3-D3,"")</f>
+        <v/>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
+      <c r="J3" s="13"/>
+      <c r="K3" s="3">
+        <f>G53</f>
+        <v>0</v>
+      </c>
+      <c r="L3" s="3">
+        <f>H53</f>
+        <v>0</v>
+      </c>
+      <c r="M3" s="3">
+        <f>I53</f>
+        <v>0</v>
+      </c>
+      <c r="N3" s="7" t="str">
+        <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
+        <v/>
+      </c>
+      <c r="O3" s="6" t="str">
+        <f>IF(B16=K3,MAX(E:E),"")</f>
+        <v/>
+      </c>
+      <c r="P3" s="2" t="str">
+        <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
+        <v/>
+      </c>
+      <c r="Q3" s="2" t="str">
+        <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
+        <v/>
+      </c>
+      <c r="T3" s="12"/>
+      <c r="X3" s="6">
+        <f>B9</f>
+        <v>46234</v>
+      </c>
+      <c r="Y3" s="3">
+        <f>B16*-1</f>
+        <v>-10.7</v>
+      </c>
+      <c r="Z3" s="2" t="str">
+        <f ca="1">IF(AND(TODAY()&gt;B11, K3&lt;&gt;B16), "+", "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="16" t="str">
+        <f>IF(E4&gt;0,E4-D4,"")</f>
+        <v/>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="9"/>
+      <c r="X4" s="6">
+        <f>E3</f>
+        <v>0</v>
+      </c>
+      <c r="Y4" s="3">
+        <f>G3+H3-I3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A5" s="5"/>
+      <c r="B5" s="6"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="16" t="str">
+        <f t="shared" ref="F5:F52" si="0">IF(E5&gt;0,E5-D5,"")</f>
+        <v/>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="9"/>
+      <c r="X5" s="6">
+        <f t="shared" ref="X5:X52" si="1">E4</f>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="3">
+        <f t="shared" ref="Y5:Y52" si="2">G4+H4-I4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A6" s="5"/>
+      <c r="B6" s="6"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="9"/>
+      <c r="X6" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y6" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A7" s="5"/>
+      <c r="B7" s="6"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="13"/>
+      <c r="X7" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y7" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="6" t="str">
+        <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
+        <v>0 m. 2 mėn. 12 d.</v>
+      </c>
+      <c r="D8" s="10"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="9"/>
+      <c r="X8" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y8" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="6">
+        <v>46234</v>
+      </c>
+      <c r="D9" s="10"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="13"/>
+      <c r="X9" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y9" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="6">
+        <v>46128</v>
+      </c>
+      <c r="D10" s="10"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="13"/>
+      <c r="X10" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y10" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="6">
+        <v>46308</v>
+      </c>
+      <c r="D11" s="10"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="13"/>
+      <c r="X11" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y11" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="16">
+        <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
+        <v>73</v>
+      </c>
+      <c r="D12" s="10"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="13"/>
+      <c r="X12" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y12" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A13" s="5"/>
+      <c r="B13" s="3"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="13"/>
+      <c r="N13" s="12"/>
+      <c r="X13" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y13" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="22"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="13"/>
+      <c r="X14" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y14" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="7">
+        <v>0.15</v>
+      </c>
+      <c r="D15" s="10"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="18"/>
+      <c r="M15" s="18"/>
+      <c r="N15" s="18"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="18"/>
+      <c r="Q15" s="18"/>
+      <c r="X15" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y15" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="3">
+        <v>10.7</v>
+      </c>
+      <c r="D16" s="10"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="19"/>
+      <c r="O16" s="20"/>
+      <c r="P16" s="13"/>
+      <c r="Q16" s="13"/>
+      <c r="X16" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y16" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D17" s="10"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="13"/>
+      <c r="X17" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y17" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D18" s="10"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="13"/>
+      <c r="X18" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y18" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D19" s="10"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="13"/>
+      <c r="X19" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y19" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D20" s="10"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="13"/>
+      <c r="X20" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y20" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D21" s="10"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="13"/>
+      <c r="X21" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y21" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D22" s="10"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="13"/>
+      <c r="X22" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y22" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D23" s="10"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="13"/>
+      <c r="X23" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y23" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D24" s="10"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="13"/>
+      <c r="X24" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y24" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D25" s="10"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="13"/>
+      <c r="X25" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y25" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D26" s="10"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="13"/>
+      <c r="X26" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y26" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D27" s="10"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="13"/>
+      <c r="X27" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y27" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D28" s="10"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="13"/>
+      <c r="X28" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y28" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D29" s="10"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="13"/>
+      <c r="X29" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y29" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D30" s="10"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="13"/>
+      <c r="X30" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y30" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D31" s="10"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="13"/>
+      <c r="X31" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y31" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D32" s="10"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="13"/>
+      <c r="X32" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y32" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D33" s="10"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="13"/>
+      <c r="X33" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y33" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D34" s="10"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="13"/>
+      <c r="X34" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y34" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D35" s="10"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="13"/>
+      <c r="X35" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y35" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D36" s="10"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="13"/>
+      <c r="X36" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y36" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D37" s="10"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="13"/>
+      <c r="X37" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y37" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D38" s="10"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="13"/>
+      <c r="X38" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y38" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D39" s="10"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="13"/>
+      <c r="X39" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y39" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D40" s="10"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="13"/>
+      <c r="X40" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y40" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D41" s="10"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="13"/>
+      <c r="X41" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y41" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D42" s="10"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="13"/>
+      <c r="X42" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y42" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D43" s="10"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
+      <c r="J43" s="13"/>
+      <c r="X43" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y43" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D44" s="10"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="13"/>
+      <c r="X44" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y44" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D45" s="10"/>
+      <c r="E45" s="6"/>
+      <c r="F45" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="13"/>
+      <c r="X45" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y45" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D46" s="10"/>
+      <c r="E46" s="6"/>
+      <c r="F46" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2"/>
+      <c r="J46" s="13"/>
+      <c r="X46" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y46" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D47" s="10"/>
+      <c r="E47" s="6"/>
+      <c r="F47" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+      <c r="J47" s="13"/>
+      <c r="X47" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y47" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D48" s="10"/>
+      <c r="E48" s="6"/>
+      <c r="F48" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="13"/>
+      <c r="X48" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y48" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D49" s="10"/>
+      <c r="E49" s="6"/>
+      <c r="F49" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
+      <c r="I49" s="2"/>
+      <c r="J49" s="13"/>
+      <c r="X49" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y49" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D50" s="10"/>
+      <c r="E50" s="6"/>
+      <c r="F50" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
+      <c r="I50" s="2"/>
+      <c r="J50" s="13"/>
+      <c r="X50" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y50" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D51" s="10"/>
+      <c r="E51" s="6"/>
+      <c r="F51" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="13"/>
+      <c r="X51" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y51" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D52" s="10"/>
+      <c r="E52" s="6"/>
+      <c r="F52" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="9"/>
+      <c r="X52" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y52" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D53" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E53" s="23"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3">
+        <f>SUM(G3:G52)</f>
+        <v>0</v>
+      </c>
+      <c r="H53" s="3">
+        <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
+        <v>0</v>
+      </c>
+      <c r="I53" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="K1:Q1"/>
+    <mergeCell ref="X1:Z1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1:B1">
+    <cfRule type="expression" dxfId="55" priority="1">
+      <formula>$Z$3="+"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="54" priority="2">
+      <formula>$B$16=$K$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P3">
+    <cfRule type="expression" dxfId="53" priority="3">
+      <formula>$Z$3="+"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z3">
+    <cfRule type="expression" dxfId="52" priority="4">
+      <formula>$Z$3="+"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C4D5F6A-B14E-4785-B9AF-25A52B6D4EFA}">
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12723,22 +15448,30 @@
       <c r="D3" s="10">
         <v>46234</v>
       </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="16" t="str">
+      <c r="E3" s="10">
+        <v>46233</v>
+      </c>
+      <c r="F3" s="16">
         <f>IF(E3&gt;0,E3-D3,"")</f>
-        <v/>
-      </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+        <v>-1</v>
+      </c>
+      <c r="G3" s="3">
+        <v>1.01</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
       <c r="J3" s="13"/>
       <c r="K3" s="3">
         <f>G53</f>
-        <v>0</v>
+        <v>1.01</v>
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
@@ -12781,7 +15514,9 @@
       <c r="B4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="10"/>
+      <c r="D4" s="10">
+        <v>46265</v>
+      </c>
       <c r="E4" s="10"/>
       <c r="F4" s="16" t="str">
         <f>IF(E4&gt;0,E4-D4,"")</f>
@@ -12793,11 +15528,11 @@
       <c r="J4" s="9"/>
       <c r="X4" s="6">
         <f>E3</f>
-        <v>0</v>
+        <v>46233</v>
       </c>
       <c r="Y4" s="3">
         <f>G3+H3-I3</f>
-        <v>0</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
@@ -12977,7 +15712,7 @@
       </c>
       <c r="B12" s="16">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -13837,11 +16572,11 @@
       <c r="F53" s="3"/>
       <c r="G53" s="3">
         <f>SUM(G3:G52)</f>
-        <v>0</v>
+        <v>1.01</v>
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
@@ -13879,7 +16614,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D992D7B8-930F-4AFA-8660-FCBCA926F777}">
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14063,7 +16798,9 @@
       <c r="B4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="10"/>
+      <c r="D4" s="10">
+        <v>46262</v>
+      </c>
       <c r="E4" s="10"/>
       <c r="F4" s="16" t="str">
         <f>IF(E4&gt;0,E4-D4,"")</f>
@@ -14259,7 +16996,7 @@
       </c>
       <c r="B12" s="16">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -15161,7 +17898,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05A12BF4-C04E-4220-8B17-E9AD0A5D2907}">
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -15543,7 +18280,7 @@
       </c>
       <c r="B12" s="16">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>1242</v>
+        <v>1239</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -16445,7 +19182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32E34830-067C-4069-8BB5-3E33A8AAE3C5}">
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -16596,7 +19333,7 @@
       </c>
       <c r="P3" s="2">
         <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="Q3" s="2" t="str">
         <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
@@ -16819,7 +19556,7 @@
       </c>
       <c r="B12" s="16">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>-6</v>
+        <v>-9</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -17721,7 +20458,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3EED607-E3C3-46C6-8528-B40D7AA70A10}">
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -18093,7 +20830,7 @@
       </c>
       <c r="B12" s="16">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -18995,7 +21732,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D504CDC9-F42B-41A7-926F-D0C0266DA0F7}">
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -19132,11 +21869,11 @@
       <c r="J3" s="13"/>
       <c r="K3" s="3">
         <f>G53</f>
-        <v>3.19</v>
+        <v>6.41</v>
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.05</v>
+        <v>0.13</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
@@ -19180,16 +21917,24 @@
         <v>31</v>
       </c>
       <c r="D4" s="10">
-        <v>46234</v>
-      </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="16" t="str">
+        <v>46233</v>
+      </c>
+      <c r="E4" s="10">
+        <v>46233</v>
+      </c>
+      <c r="F4" s="16">
         <f>IF(E4&gt;0,E4-D4,"")</f>
-        <v/>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="3"/>
+        <v>0</v>
+      </c>
+      <c r="G4" s="3">
+        <v>3.22</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0.08</v>
+      </c>
+      <c r="I4" s="3">
+        <v>0</v>
+      </c>
       <c r="J4" s="9"/>
       <c r="X4" s="6">
         <f>E3</f>
@@ -19215,11 +21960,11 @@
       <c r="J5" s="9"/>
       <c r="X5" s="6">
         <f t="shared" ref="X5:X52" si="1">E4</f>
-        <v>0</v>
+        <v>46233</v>
       </c>
       <c r="Y5" s="3">
         <f t="shared" ref="Y5:Y52" si="2">G4+H4-I4</f>
-        <v>0</v>
+        <v>3.3000000000000003</v>
       </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
@@ -19377,7 +22122,7 @@
       </c>
       <c r="B12" s="16">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -20237,11 +22982,11 @@
       <c r="F53" s="3"/>
       <c r="G53" s="3">
         <f>SUM(G3:G52)</f>
-        <v>3.19</v>
+        <v>6.41</v>
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.05</v>
+        <v>0.13</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
@@ -20277,1309 +23022,4 @@
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{615F6B81-524E-46B8-96DD-07557B282857}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
-  <dimension ref="A1:Z53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="40.7109375" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" customWidth="1"/>
-    <col min="4" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="9" width="10.7109375" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" customWidth="1"/>
-    <col min="11" max="14" width="10.7109375" customWidth="1"/>
-    <col min="15" max="15" width="12.7109375" customWidth="1"/>
-    <col min="16" max="17" width="10.7109375" customWidth="1"/>
-    <col min="18" max="23" width="8.7109375" customWidth="1"/>
-    <col min="24" max="24" width="12.7109375" style="13" customWidth="1"/>
-    <col min="25" max="25" width="10.7109375" style="13" customWidth="1"/>
-    <col min="26" max="26" width="10.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" s="32" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="32" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="33"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33"/>
-      <c r="N1" s="33"/>
-      <c r="O1" s="33"/>
-      <c r="P1" s="33"/>
-      <c r="Q1" s="34"/>
-      <c r="X1" s="32"/>
-      <c r="Y1" s="33"/>
-      <c r="Z1" s="34"/>
-    </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="J2" s="9"/>
-      <c r="K2" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="L2" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="M2" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="N2" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="O2" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="P2" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q2" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="X2" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="Y2" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z2" s="11" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D3" s="10">
-        <v>46172</v>
-      </c>
-      <c r="E3" s="10">
-        <v>46174</v>
-      </c>
-      <c r="F3" s="16">
-        <f>IF(E3&gt;0,E3-D3,"")</f>
-        <v>2</v>
-      </c>
-      <c r="G3" s="3">
-        <v>1.1599999999999999</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0.01</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
-      <c r="J3" s="13"/>
-      <c r="K3" s="3">
-        <f>G53</f>
-        <v>12.809999999999999</v>
-      </c>
-      <c r="L3" s="3">
-        <f>H53</f>
-        <v>0.11</v>
-      </c>
-      <c r="M3" s="3">
-        <f>I53</f>
-        <v>0</v>
-      </c>
-      <c r="N3" s="7">
-        <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
-        <v>0.11385952830314636</v>
-      </c>
-      <c r="O3" s="6">
-        <f>IF(B16=K3,MAX(E:E),"")</f>
-        <v>46205</v>
-      </c>
-      <c r="P3" s="2" t="str">
-        <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
-        <v/>
-      </c>
-      <c r="Q3" s="2">
-        <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
-        <v>-271</v>
-      </c>
-      <c r="T3" s="12"/>
-      <c r="X3" s="6">
-        <f>B9</f>
-        <v>46169</v>
-      </c>
-      <c r="Y3" s="3">
-        <f>B16*-1</f>
-        <v>-12.81</v>
-      </c>
-      <c r="Z3" s="2" t="str">
-        <f ca="1">IF(AND(TODAY()&gt;B11, K3&lt;&gt;B16), "+", "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" s="10">
-        <v>46203</v>
-      </c>
-      <c r="E4" s="10">
-        <v>46175</v>
-      </c>
-      <c r="F4" s="16">
-        <f>IF(E4&gt;0,E4-D4,"")</f>
-        <v>-28</v>
-      </c>
-      <c r="G4" s="3">
-        <v>1.81</v>
-      </c>
-      <c r="H4" s="2">
-        <v>0.01</v>
-      </c>
-      <c r="I4" s="3">
-        <v>0</v>
-      </c>
-      <c r="J4" s="9"/>
-      <c r="X4" s="6">
-        <f>E3</f>
-        <v>46174</v>
-      </c>
-      <c r="Y4" s="3">
-        <f>G3+H3-I3</f>
-        <v>1.17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6"/>
-      <c r="D5" s="10">
-        <v>46233</v>
-      </c>
-      <c r="E5" s="10">
-        <v>46205</v>
-      </c>
-      <c r="F5" s="16">
-        <f t="shared" ref="F5:F52" si="0">IF(E5&gt;0,E5-D5,"")</f>
-        <v>-28</v>
-      </c>
-      <c r="G5" s="3">
-        <v>9.84</v>
-      </c>
-      <c r="H5" s="3">
-        <v>0.09</v>
-      </c>
-      <c r="I5" s="3">
-        <v>0</v>
-      </c>
-      <c r="J5" s="9"/>
-      <c r="X5" s="6">
-        <f t="shared" ref="X5:X52" si="1">E4</f>
-        <v>46175</v>
-      </c>
-      <c r="Y5" s="3">
-        <f t="shared" ref="Y5:Y52" si="2">G4+H4-I4</f>
-        <v>1.82</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A6" s="5"/>
-      <c r="B6" s="6"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="9"/>
-      <c r="X6" s="6">
-        <f t="shared" si="1"/>
-        <v>46205</v>
-      </c>
-      <c r="Y6" s="3">
-        <f t="shared" si="2"/>
-        <v>9.93</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="13"/>
-      <c r="X7" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y7" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="6" t="str">
-        <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
-        <v>0 m. 10 mėn. 3 d.</v>
-      </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="9"/>
-      <c r="X8" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y8" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="6">
-        <v>46169</v>
-      </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="13"/>
-      <c r="X9" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y9" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="6">
-        <v>46108</v>
-      </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="13"/>
-      <c r="X10" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y10" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="6">
-        <v>46476</v>
-      </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="13"/>
-      <c r="X11" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y11" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B12" s="16" t="str">
-        <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v/>
-      </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="13"/>
-      <c r="X12" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y12" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A13" s="5"/>
-      <c r="B13" s="3"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="13"/>
-      <c r="N13" s="12"/>
-      <c r="X13" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y13" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="22"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="13"/>
-      <c r="X14" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y14" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="7">
-        <v>0.11</v>
-      </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="18"/>
-      <c r="M15" s="18"/>
-      <c r="N15" s="18"/>
-      <c r="O15" s="18"/>
-      <c r="P15" s="18"/>
-      <c r="Q15" s="18"/>
-      <c r="X15" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y15" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B16" s="3">
-        <v>12.81</v>
-      </c>
-      <c r="D16" s="10"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="19"/>
-      <c r="O16" s="20"/>
-      <c r="P16" s="13"/>
-      <c r="Q16" s="13"/>
-      <c r="X16" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y16" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D17" s="10"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="13"/>
-      <c r="X17" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y17" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D18" s="10"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="13"/>
-      <c r="X18" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y18" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D19" s="10"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="13"/>
-      <c r="X19" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y19" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D20" s="10"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="13"/>
-      <c r="X20" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y20" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D21" s="10"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="13"/>
-      <c r="X21" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y21" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D22" s="10"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="13"/>
-      <c r="X22" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y22" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D23" s="10"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="13"/>
-      <c r="X23" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y23" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D24" s="10"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="13"/>
-      <c r="X24" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y24" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D25" s="10"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="13"/>
-      <c r="X25" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y25" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D26" s="10"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="13"/>
-      <c r="X26" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y26" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D27" s="10"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="13"/>
-      <c r="X27" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y27" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D28" s="10"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="13"/>
-      <c r="X28" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y28" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D29" s="10"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="13"/>
-      <c r="X29" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y29" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D30" s="10"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="13"/>
-      <c r="X30" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y30" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D31" s="10"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="13"/>
-      <c r="X31" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y31" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D32" s="10"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="13"/>
-      <c r="X32" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y32" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D33" s="10"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="13"/>
-      <c r="X33" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y33" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D34" s="10"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="13"/>
-      <c r="X34" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y34" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D35" s="10"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-      <c r="J35" s="13"/>
-      <c r="X35" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y35" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D36" s="10"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="13"/>
-      <c r="X36" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y36" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D37" s="10"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="13"/>
-      <c r="X37" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y37" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D38" s="10"/>
-      <c r="E38" s="6"/>
-      <c r="F38" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="13"/>
-      <c r="X38" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y38" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D39" s="10"/>
-      <c r="E39" s="6"/>
-      <c r="F39" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G39" s="2"/>
-      <c r="H39" s="2"/>
-      <c r="I39" s="2"/>
-      <c r="J39" s="13"/>
-      <c r="X39" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y39" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D40" s="10"/>
-      <c r="E40" s="6"/>
-      <c r="F40" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
-      <c r="J40" s="13"/>
-      <c r="X40" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y40" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D41" s="10"/>
-      <c r="E41" s="6"/>
-      <c r="F41" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G41" s="2"/>
-      <c r="H41" s="2"/>
-      <c r="I41" s="2"/>
-      <c r="J41" s="13"/>
-      <c r="X41" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y41" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D42" s="10"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G42" s="2"/>
-      <c r="H42" s="2"/>
-      <c r="I42" s="2"/>
-      <c r="J42" s="13"/>
-      <c r="X42" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y42" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D43" s="10"/>
-      <c r="E43" s="6"/>
-      <c r="F43" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G43" s="2"/>
-      <c r="H43" s="2"/>
-      <c r="I43" s="2"/>
-      <c r="J43" s="13"/>
-      <c r="X43" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y43" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D44" s="10"/>
-      <c r="E44" s="6"/>
-      <c r="F44" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G44" s="2"/>
-      <c r="H44" s="2"/>
-      <c r="I44" s="2"/>
-      <c r="J44" s="13"/>
-      <c r="X44" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y44" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D45" s="10"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="13"/>
-      <c r="X45" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y45" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D46" s="10"/>
-      <c r="E46" s="6"/>
-      <c r="F46" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G46" s="2"/>
-      <c r="H46" s="2"/>
-      <c r="I46" s="2"/>
-      <c r="J46" s="13"/>
-      <c r="X46" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y46" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D47" s="10"/>
-      <c r="E47" s="6"/>
-      <c r="F47" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G47" s="2"/>
-      <c r="H47" s="2"/>
-      <c r="I47" s="2"/>
-      <c r="J47" s="13"/>
-      <c r="X47" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y47" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D48" s="10"/>
-      <c r="E48" s="6"/>
-      <c r="F48" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G48" s="2"/>
-      <c r="H48" s="2"/>
-      <c r="I48" s="2"/>
-      <c r="J48" s="13"/>
-      <c r="X48" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y48" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D49" s="10"/>
-      <c r="E49" s="6"/>
-      <c r="F49" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G49" s="2"/>
-      <c r="H49" s="2"/>
-      <c r="I49" s="2"/>
-      <c r="J49" s="13"/>
-      <c r="X49" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y49" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D50" s="10"/>
-      <c r="E50" s="6"/>
-      <c r="F50" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G50" s="2"/>
-      <c r="H50" s="2"/>
-      <c r="I50" s="2"/>
-      <c r="J50" s="13"/>
-      <c r="X50" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y50" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D51" s="10"/>
-      <c r="E51" s="6"/>
-      <c r="F51" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
-      <c r="I51" s="2"/>
-      <c r="J51" s="13"/>
-      <c r="X51" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y51" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D52" s="10"/>
-      <c r="E52" s="6"/>
-      <c r="F52" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
-      <c r="I52" s="2"/>
-      <c r="J52" s="9"/>
-      <c r="X52" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y52" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="4:25" x14ac:dyDescent="0.25">
-      <c r="D53" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E53" s="23"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="3">
-        <f>SUM(G3:G52)</f>
-        <v>12.809999999999999</v>
-      </c>
-      <c r="H53" s="3">
-        <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.11</v>
-      </c>
-      <c r="I53" s="3">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="K1:Q1"/>
-    <mergeCell ref="X1:Z1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="27" priority="1">
-      <formula>$Z$3="+"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="26" priority="2">
-      <formula>$B$16=$K$3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="25" priority="5">
-      <formula>$Z$3="+"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="24" priority="6">
-      <formula>$Z$3="+"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
 </file>
</xml_diff>